<commit_message>
curriculum: publish v0.3 complex-number scope split
</commit_message>
<xml_diff>
--- a/curriculum/master-map/Mathematics_Understood_Master_Curriculum_Map_v0.3.xlsx
+++ b/curriculum/master-map/Mathematics_Understood_Master_Curriculum_Map_v0.3.xlsx
@@ -759,7 +759,7 @@
     <tableColumn id="7" name="v0.3 preliminary review classification"/>
     <tableColumn id="8" name="Specific dependency mechanism / evidence"/>
     <tableColumn id="9" name="Proposed validation check / test"/>
-    <tableColumn id="10" name="Reviewer"/>
+    <tableColumn id="10" name="Reviewer / provenance"/>
     <tableColumn id="11" name="Review date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -20426,7 +20426,7 @@
       </c>
       <c r="J4" s="74" t="inlineStr">
         <is>
-          <t>Reviewer</t>
+          <t>Reviewer / provenance</t>
         </is>
       </c>
       <c r="K4" s="74" t="inlineStr">

</xml_diff>